<commit_message>
band-advance: regenerate clean advance-list template (purge test data)
Pilot proved out; wiped all test data (DB tables, uploads, disk records, the
filed FSQ test tree) and reset the sheet to a fresh no-data template from
build_template.py.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Advancing/_template/advance-list-template.xlsx
+++ b/Advancing/_template/advance-list-template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Advance List" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_lists" sheetId="2" state="hidden" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Advance List" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="_lists" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -731,113 +731,41 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>513 Airwaves w/ Inhailer Radio</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Fountain Square</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>513 Airwaves w/ Inhailer Radio</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Internal</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>INHAILER RADIO</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>Sam</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>5136214400</t>
-        </is>
-      </c>
-      <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>4:30pm</t>
-        </is>
-      </c>
-      <c r="L3" s="5" t="inlineStr">
-        <is>
-          <t>5:00pm</t>
-        </is>
-      </c>
-      <c r="M3" s="5" t="inlineStr">
-        <is>
-          <t>9pm</t>
-        </is>
-      </c>
-      <c r="N3" s="5" t="inlineStr">
-        <is>
-          <t>10pm</t>
-        </is>
-      </c>
-      <c r="O3" s="5" t="inlineStr">
-        <is>
-          <t>11pm</t>
-        </is>
-      </c>
-      <c r="P3" s="5" t="inlineStr">
-        <is>
-          <t>headliner</t>
-        </is>
-      </c>
-      <c r="Q3" s="5" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="R3" s="5" t="inlineStr">
-        <is>
-          <t>Headiner Band</t>
-        </is>
-      </c>
-      <c r="S3" s="5" t="inlineStr">
-        <is>
-          <t>blloyd@3cdc.org</t>
-        </is>
-      </c>
-      <c r="T3" s="5" t="inlineStr"/>
-      <c r="U3" s="5" t="inlineStr"/>
-      <c r="V3" s="5" t="inlineStr"/>
-      <c r="W3" s="5" t="inlineStr"/>
-      <c r="X3" s="5" t="inlineStr"/>
-      <c r="Y3" s="5" t="inlineStr"/>
-      <c r="Z3" s="5" t="inlineStr"/>
-      <c r="AA3" s="5" t="inlineStr"/>
-      <c r="AB3" s="5" t="inlineStr"/>
-      <c r="AC3" s="5" t="inlineStr"/>
-      <c r="AD3" s="5" t="inlineStr"/>
-      <c r="AE3" s="5" t="inlineStr"/>
-      <c r="AF3" s="5" t="inlineStr"/>
-      <c r="AG3" s="5" t="inlineStr"/>
-      <c r="AH3" s="5" t="inlineStr"/>
-      <c r="AI3" s="5" t="inlineStr"/>
+      <c r="A3" s="5" t="n"/>
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
+      <c r="J3" s="5" t="n"/>
+      <c r="K3" s="5" t="n"/>
+      <c r="L3" s="5" t="n"/>
+      <c r="M3" s="5" t="n"/>
+      <c r="N3" s="5" t="n"/>
+      <c r="O3" s="5" t="n"/>
+      <c r="P3" s="5" t="n"/>
+      <c r="Q3" s="5" t="n"/>
+      <c r="R3" s="5" t="n"/>
+      <c r="S3" s="5" t="n"/>
+      <c r="T3" s="5" t="n"/>
+      <c r="U3" s="5" t="n"/>
+      <c r="V3" s="5" t="n"/>
+      <c r="W3" s="5" t="n"/>
+      <c r="X3" s="5" t="n"/>
+      <c r="Y3" s="5" t="n"/>
+      <c r="Z3" s="5" t="n"/>
+      <c r="AA3" s="5" t="n"/>
+      <c r="AB3" s="5" t="n"/>
+      <c r="AC3" s="5" t="n"/>
+      <c r="AD3" s="5" t="n"/>
+      <c r="AE3" s="5" t="n"/>
+      <c r="AF3" s="5" t="n"/>
+      <c r="AG3" s="5" t="n"/>
+      <c r="AH3" s="5" t="n"/>
+      <c r="AI3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="n"/>

</xml_diff>

<commit_message>
band-advance: venue-correct email bodies + per-artist personal note
The advance email was hardcoded to Fountain Square (garage QR codes, 95 dB
ordinance, FSQ engineer) — wrong for any other venue. Split the body into a
venue-keyed engine:

- venue_email.py: per-venue blocks (location, load-in, technical, hospitality,
  venue-only rules) + shared COMMON_REQUIREMENTS. FSQ fully wired; other venues
  fall back to safe generic blocks (no FSQ specifics) until Brian supplies copy.
- advance.md.j2 renders {{ blocks.* }} instead of baked FSQ prose.
- Per-artist "Email Note" column (fieldspec ACT_FIELDS): whatever Brian types per
  show is woven into that band's draft as a personal paragraph; omitted cleanly
  when blank.

Verified: an FSQ draft carries garage/95 dB + the note; a Washington Park draft
gets generic load-in with none of the FSQ specifics and no note.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Advancing/_template/advance-list-template.xlsx
+++ b/Advancing/_template/advance-list-template.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI200"/>
+  <dimension ref="A1:AJ200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -524,16 +524,17 @@
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="14" customWidth="1" min="24" max="24"/>
     <col width="14" customWidth="1" min="25" max="25"/>
-    <col width="26" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
     <col width="26" customWidth="1" min="27" max="27"/>
     <col width="26" customWidth="1" min="28" max="28"/>
-    <col width="14" customWidth="1" min="29" max="29"/>
-    <col width="26" customWidth="1" min="30" max="30"/>
+    <col width="26" customWidth="1" min="29" max="29"/>
+    <col width="14" customWidth="1" min="30" max="30"/>
     <col width="26" customWidth="1" min="31" max="31"/>
-    <col width="14" customWidth="1" min="32" max="32"/>
+    <col width="26" customWidth="1" min="32" max="32"/>
     <col width="14" customWidth="1" min="33" max="33"/>
     <col width="14" customWidth="1" min="34" max="34"/>
     <col width="14" customWidth="1" min="35" max="35"/>
+    <col width="14" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -547,7 +548,7 @@
           <t>ACT</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>BAND DETAILS — usually from the form; fill to override</t>
         </is>
@@ -651,80 +652,85 @@
       </c>
       <c r="T2" s="4" t="inlineStr">
         <is>
+          <t>Email Note</t>
+        </is>
+      </c>
+      <c r="U2" s="4" t="inlineStr">
+        <is>
           <t>Contact Name</t>
         </is>
       </c>
-      <c r="U2" s="4" t="inlineStr">
+      <c r="V2" s="4" t="inlineStr">
         <is>
           <t>Contact Phone</t>
         </is>
       </c>
-      <c r="V2" s="4" t="inlineStr">
+      <c r="W2" s="4" t="inlineStr">
         <is>
           <t>Stage Type</t>
         </is>
       </c>
-      <c r="W2" s="4" t="inlineStr">
+      <c r="X2" s="4" t="inlineStr">
         <is>
           <t>Monitors</t>
         </is>
       </c>
-      <c r="X2" s="4" t="inlineStr">
+      <c r="Y2" s="4" t="inlineStr">
         <is>
           <t>Own IEMs</t>
         </is>
       </c>
-      <c r="Y2" s="4" t="inlineStr">
+      <c r="Z2" s="4" t="inlineStr">
         <is>
           <t>Split Snake</t>
         </is>
       </c>
-      <c r="Z2" s="4" t="inlineStr">
+      <c r="AA2" s="4" t="inlineStr">
         <is>
           <t>Stage Plot</t>
         </is>
       </c>
-      <c r="AA2" s="4" t="inlineStr">
+      <c r="AB2" s="4" t="inlineStr">
         <is>
           <t>Input Notes</t>
         </is>
       </c>
-      <c r="AB2" s="4" t="inlineStr">
+      <c r="AC2" s="4" t="inlineStr">
         <is>
           <t>Backline</t>
         </is>
       </c>
-      <c r="AC2" s="4" t="inlineStr">
+      <c r="AD2" s="4" t="inlineStr">
         <is>
           <t>Own Engineer</t>
         </is>
       </c>
-      <c r="AD2" s="4" t="inlineStr">
+      <c r="AE2" s="4" t="inlineStr">
         <is>
           <t>Scenic</t>
         </is>
       </c>
-      <c r="AE2" s="4" t="inlineStr">
+      <c r="AF2" s="4" t="inlineStr">
         <is>
           <t>Lighting</t>
         </is>
       </c>
-      <c r="AF2" s="4" t="inlineStr">
+      <c r="AG2" s="4" t="inlineStr">
         <is>
           <t>Merch</t>
         </is>
       </c>
-      <c r="AG2" s="4" t="inlineStr">
+      <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>Band Tent</t>
         </is>
       </c>
-      <c r="AH2" s="4" t="inlineStr">
+      <c r="AI2" s="4" t="inlineStr">
         <is>
           <t>Performers</t>
         </is>
       </c>
-      <c r="AI2" s="4" t="inlineStr">
+      <c r="AJ2" s="4" t="inlineStr">
         <is>
           <t>Large Vehicle</t>
         </is>
@@ -766,6 +772,7 @@
       <c r="AG3" s="5" t="n"/>
       <c r="AH3" s="5" t="n"/>
       <c r="AI3" s="5" t="n"/>
+      <c r="AJ3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="n"/>
@@ -803,6 +810,7 @@
       <c r="AG4" s="6" t="n"/>
       <c r="AH4" s="6" t="n"/>
       <c r="AI4" s="6" t="n"/>
+      <c r="AJ4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n"/>
@@ -840,6 +848,7 @@
       <c r="AG5" s="5" t="n"/>
       <c r="AH5" s="5" t="n"/>
       <c r="AI5" s="5" t="n"/>
+      <c r="AJ5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n"/>
@@ -877,6 +886,7 @@
       <c r="AG6" s="6" t="n"/>
       <c r="AH6" s="6" t="n"/>
       <c r="AI6" s="6" t="n"/>
+      <c r="AJ6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n"/>
@@ -914,6 +924,7 @@
       <c r="AG7" s="5" t="n"/>
       <c r="AH7" s="5" t="n"/>
       <c r="AI7" s="5" t="n"/>
+      <c r="AJ7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n"/>
@@ -951,6 +962,7 @@
       <c r="AG8" s="6" t="n"/>
       <c r="AH8" s="6" t="n"/>
       <c r="AI8" s="6" t="n"/>
+      <c r="AJ8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
@@ -988,6 +1000,7 @@
       <c r="AG9" s="5" t="n"/>
       <c r="AH9" s="5" t="n"/>
       <c r="AI9" s="5" t="n"/>
+      <c r="AJ9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
@@ -1025,6 +1038,7 @@
       <c r="AG10" s="6" t="n"/>
       <c r="AH10" s="6" t="n"/>
       <c r="AI10" s="6" t="n"/>
+      <c r="AJ10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
@@ -1062,6 +1076,7 @@
       <c r="AG11" s="5" t="n"/>
       <c r="AH11" s="5" t="n"/>
       <c r="AI11" s="5" t="n"/>
+      <c r="AJ11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n"/>
@@ -1099,6 +1114,7 @@
       <c r="AG12" s="6" t="n"/>
       <c r="AH12" s="6" t="n"/>
       <c r="AI12" s="6" t="n"/>
+      <c r="AJ12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
@@ -1136,6 +1152,7 @@
       <c r="AG13" s="5" t="n"/>
       <c r="AH13" s="5" t="n"/>
       <c r="AI13" s="5" t="n"/>
+      <c r="AJ13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
@@ -1173,6 +1190,7 @@
       <c r="AG14" s="6" t="n"/>
       <c r="AH14" s="6" t="n"/>
       <c r="AI14" s="6" t="n"/>
+      <c r="AJ14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
@@ -1210,6 +1228,7 @@
       <c r="AG15" s="5" t="n"/>
       <c r="AH15" s="5" t="n"/>
       <c r="AI15" s="5" t="n"/>
+      <c r="AJ15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n"/>
@@ -1247,6 +1266,7 @@
       <c r="AG16" s="6" t="n"/>
       <c r="AH16" s="6" t="n"/>
       <c r="AI16" s="6" t="n"/>
+      <c r="AJ16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
@@ -1284,6 +1304,7 @@
       <c r="AG17" s="5" t="n"/>
       <c r="AH17" s="5" t="n"/>
       <c r="AI17" s="5" t="n"/>
+      <c r="AJ17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
@@ -1321,6 +1342,7 @@
       <c r="AG18" s="6" t="n"/>
       <c r="AH18" s="6" t="n"/>
       <c r="AI18" s="6" t="n"/>
+      <c r="AJ18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
@@ -1358,6 +1380,7 @@
       <c r="AG19" s="5" t="n"/>
       <c r="AH19" s="5" t="n"/>
       <c r="AI19" s="5" t="n"/>
+      <c r="AJ19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n"/>
@@ -1395,6 +1418,7 @@
       <c r="AG20" s="6" t="n"/>
       <c r="AH20" s="6" t="n"/>
       <c r="AI20" s="6" t="n"/>
+      <c r="AJ20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n"/>
@@ -1432,6 +1456,7 @@
       <c r="AG21" s="5" t="n"/>
       <c r="AH21" s="5" t="n"/>
       <c r="AI21" s="5" t="n"/>
+      <c r="AJ21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n"/>
@@ -1469,6 +1494,7 @@
       <c r="AG22" s="6" t="n"/>
       <c r="AH22" s="6" t="n"/>
       <c r="AI22" s="6" t="n"/>
+      <c r="AJ22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n"/>
@@ -1506,6 +1532,7 @@
       <c r="AG23" s="5" t="n"/>
       <c r="AH23" s="5" t="n"/>
       <c r="AI23" s="5" t="n"/>
+      <c r="AJ23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n"/>
@@ -1543,6 +1570,7 @@
       <c r="AG24" s="6" t="n"/>
       <c r="AH24" s="6" t="n"/>
       <c r="AI24" s="6" t="n"/>
+      <c r="AJ24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n"/>
@@ -1580,6 +1608,7 @@
       <c r="AG25" s="5" t="n"/>
       <c r="AH25" s="5" t="n"/>
       <c r="AI25" s="5" t="n"/>
+      <c r="AJ25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n"/>
@@ -1617,6 +1646,7 @@
       <c r="AG26" s="6" t="n"/>
       <c r="AH26" s="6" t="n"/>
       <c r="AI26" s="6" t="n"/>
+      <c r="AJ26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n"/>
@@ -1654,6 +1684,7 @@
       <c r="AG27" s="5" t="n"/>
       <c r="AH27" s="5" t="n"/>
       <c r="AI27" s="5" t="n"/>
+      <c r="AJ27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n"/>
@@ -1691,6 +1722,7 @@
       <c r="AG28" s="6" t="n"/>
       <c r="AH28" s="6" t="n"/>
       <c r="AI28" s="6" t="n"/>
+      <c r="AJ28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n"/>
@@ -1728,6 +1760,7 @@
       <c r="AG29" s="5" t="n"/>
       <c r="AH29" s="5" t="n"/>
       <c r="AI29" s="5" t="n"/>
+      <c r="AJ29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n"/>
@@ -1765,6 +1798,7 @@
       <c r="AG30" s="6" t="n"/>
       <c r="AH30" s="6" t="n"/>
       <c r="AI30" s="6" t="n"/>
+      <c r="AJ30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n"/>
@@ -1802,6 +1836,7 @@
       <c r="AG31" s="5" t="n"/>
       <c r="AH31" s="5" t="n"/>
       <c r="AI31" s="5" t="n"/>
+      <c r="AJ31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n"/>
@@ -1839,6 +1874,7 @@
       <c r="AG32" s="6" t="n"/>
       <c r="AH32" s="6" t="n"/>
       <c r="AI32" s="6" t="n"/>
+      <c r="AJ32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n"/>
@@ -1876,6 +1912,7 @@
       <c r="AG33" s="5" t="n"/>
       <c r="AH33" s="5" t="n"/>
       <c r="AI33" s="5" t="n"/>
+      <c r="AJ33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n"/>
@@ -1913,6 +1950,7 @@
       <c r="AG34" s="6" t="n"/>
       <c r="AH34" s="6" t="n"/>
       <c r="AI34" s="6" t="n"/>
+      <c r="AJ34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n"/>
@@ -1950,6 +1988,7 @@
       <c r="AG35" s="5" t="n"/>
       <c r="AH35" s="5" t="n"/>
       <c r="AI35" s="5" t="n"/>
+      <c r="AJ35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n"/>
@@ -1987,6 +2026,7 @@
       <c r="AG36" s="6" t="n"/>
       <c r="AH36" s="6" t="n"/>
       <c r="AI36" s="6" t="n"/>
+      <c r="AJ36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n"/>
@@ -2024,6 +2064,7 @@
       <c r="AG37" s="5" t="n"/>
       <c r="AH37" s="5" t="n"/>
       <c r="AI37" s="5" t="n"/>
+      <c r="AJ37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n"/>
@@ -2061,6 +2102,7 @@
       <c r="AG38" s="6" t="n"/>
       <c r="AH38" s="6" t="n"/>
       <c r="AI38" s="6" t="n"/>
+      <c r="AJ38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n"/>
@@ -2098,6 +2140,7 @@
       <c r="AG39" s="5" t="n"/>
       <c r="AH39" s="5" t="n"/>
       <c r="AI39" s="5" t="n"/>
+      <c r="AJ39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n"/>
@@ -2135,6 +2178,7 @@
       <c r="AG40" s="6" t="n"/>
       <c r="AH40" s="6" t="n"/>
       <c r="AI40" s="6" t="n"/>
+      <c r="AJ40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n"/>
@@ -2172,6 +2216,7 @@
       <c r="AG41" s="5" t="n"/>
       <c r="AH41" s="5" t="n"/>
       <c r="AI41" s="5" t="n"/>
+      <c r="AJ41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n"/>
@@ -2209,6 +2254,7 @@
       <c r="AG42" s="6" t="n"/>
       <c r="AH42" s="6" t="n"/>
       <c r="AI42" s="6" t="n"/>
+      <c r="AJ42" s="6" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n"/>
@@ -2246,6 +2292,7 @@
       <c r="AG43" s="5" t="n"/>
       <c r="AH43" s="5" t="n"/>
       <c r="AI43" s="5" t="n"/>
+      <c r="AJ43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n"/>
@@ -2283,6 +2330,7 @@
       <c r="AG44" s="6" t="n"/>
       <c r="AH44" s="6" t="n"/>
       <c r="AI44" s="6" t="n"/>
+      <c r="AJ44" s="6" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n"/>
@@ -2320,6 +2368,7 @@
       <c r="AG45" s="5" t="n"/>
       <c r="AH45" s="5" t="n"/>
       <c r="AI45" s="5" t="n"/>
+      <c r="AJ45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n"/>
@@ -2357,6 +2406,7 @@
       <c r="AG46" s="6" t="n"/>
       <c r="AH46" s="6" t="n"/>
       <c r="AI46" s="6" t="n"/>
+      <c r="AJ46" s="6" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n"/>
@@ -2394,6 +2444,7 @@
       <c r="AG47" s="5" t="n"/>
       <c r="AH47" s="5" t="n"/>
       <c r="AI47" s="5" t="n"/>
+      <c r="AJ47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="n"/>
@@ -2431,6 +2482,7 @@
       <c r="AG48" s="6" t="n"/>
       <c r="AH48" s="6" t="n"/>
       <c r="AI48" s="6" t="n"/>
+      <c r="AJ48" s="6" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n"/>
@@ -2468,6 +2520,7 @@
       <c r="AG49" s="5" t="n"/>
       <c r="AH49" s="5" t="n"/>
       <c r="AI49" s="5" t="n"/>
+      <c r="AJ49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="6" t="n"/>
@@ -2505,6 +2558,7 @@
       <c r="AG50" s="6" t="n"/>
       <c r="AH50" s="6" t="n"/>
       <c r="AI50" s="6" t="n"/>
+      <c r="AJ50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n"/>
@@ -2542,6 +2596,7 @@
       <c r="AG51" s="5" t="n"/>
       <c r="AH51" s="5" t="n"/>
       <c r="AI51" s="5" t="n"/>
+      <c r="AJ51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n"/>
@@ -2579,6 +2634,7 @@
       <c r="AG52" s="6" t="n"/>
       <c r="AH52" s="6" t="n"/>
       <c r="AI52" s="6" t="n"/>
+      <c r="AJ52" s="6" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n"/>
@@ -2616,6 +2672,7 @@
       <c r="AG53" s="5" t="n"/>
       <c r="AH53" s="5" t="n"/>
       <c r="AI53" s="5" t="n"/>
+      <c r="AJ53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="n"/>
@@ -2653,6 +2710,7 @@
       <c r="AG54" s="6" t="n"/>
       <c r="AH54" s="6" t="n"/>
       <c r="AI54" s="6" t="n"/>
+      <c r="AJ54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n"/>
@@ -2690,6 +2748,7 @@
       <c r="AG55" s="5" t="n"/>
       <c r="AH55" s="5" t="n"/>
       <c r="AI55" s="5" t="n"/>
+      <c r="AJ55" s="5" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="6" t="n"/>
@@ -2727,6 +2786,7 @@
       <c r="AG56" s="6" t="n"/>
       <c r="AH56" s="6" t="n"/>
       <c r="AI56" s="6" t="n"/>
+      <c r="AJ56" s="6" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n"/>
@@ -2764,6 +2824,7 @@
       <c r="AG57" s="5" t="n"/>
       <c r="AH57" s="5" t="n"/>
       <c r="AI57" s="5" t="n"/>
+      <c r="AJ57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="n"/>
@@ -2801,6 +2862,7 @@
       <c r="AG58" s="6" t="n"/>
       <c r="AH58" s="6" t="n"/>
       <c r="AI58" s="6" t="n"/>
+      <c r="AJ58" s="6" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n"/>
@@ -2838,6 +2900,7 @@
       <c r="AG59" s="5" t="n"/>
       <c r="AH59" s="5" t="n"/>
       <c r="AI59" s="5" t="n"/>
+      <c r="AJ59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n"/>
@@ -2875,6 +2938,7 @@
       <c r="AG60" s="5" t="n"/>
       <c r="AH60" s="5" t="n"/>
       <c r="AI60" s="5" t="n"/>
+      <c r="AJ60" s="5" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n"/>
@@ -2912,6 +2976,7 @@
       <c r="AG61" s="5" t="n"/>
       <c r="AH61" s="5" t="n"/>
       <c r="AI61" s="5" t="n"/>
+      <c r="AJ61" s="5" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n"/>
@@ -2949,6 +3014,7 @@
       <c r="AG62" s="5" t="n"/>
       <c r="AH62" s="5" t="n"/>
       <c r="AI62" s="5" t="n"/>
+      <c r="AJ62" s="5" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n"/>
@@ -2986,6 +3052,7 @@
       <c r="AG63" s="5" t="n"/>
       <c r="AH63" s="5" t="n"/>
       <c r="AI63" s="5" t="n"/>
+      <c r="AJ63" s="5" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n"/>
@@ -3023,6 +3090,7 @@
       <c r="AG64" s="5" t="n"/>
       <c r="AH64" s="5" t="n"/>
       <c r="AI64" s="5" t="n"/>
+      <c r="AJ64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="n"/>
@@ -3060,6 +3128,7 @@
       <c r="AG65" s="5" t="n"/>
       <c r="AH65" s="5" t="n"/>
       <c r="AI65" s="5" t="n"/>
+      <c r="AJ65" s="5" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="n"/>
@@ -3097,6 +3166,7 @@
       <c r="AG66" s="5" t="n"/>
       <c r="AH66" s="5" t="n"/>
       <c r="AI66" s="5" t="n"/>
+      <c r="AJ66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="5" t="n"/>
@@ -3134,6 +3204,7 @@
       <c r="AG67" s="5" t="n"/>
       <c r="AH67" s="5" t="n"/>
       <c r="AI67" s="5" t="n"/>
+      <c r="AJ67" s="5" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="n"/>
@@ -3171,6 +3242,7 @@
       <c r="AG68" s="5" t="n"/>
       <c r="AH68" s="5" t="n"/>
       <c r="AI68" s="5" t="n"/>
+      <c r="AJ68" s="5" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="5" t="n"/>
@@ -3208,6 +3280,7 @@
       <c r="AG69" s="5" t="n"/>
       <c r="AH69" s="5" t="n"/>
       <c r="AI69" s="5" t="n"/>
+      <c r="AJ69" s="5" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="5" t="n"/>
@@ -3245,6 +3318,7 @@
       <c r="AG70" s="5" t="n"/>
       <c r="AH70" s="5" t="n"/>
       <c r="AI70" s="5" t="n"/>
+      <c r="AJ70" s="5" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="5" t="n"/>
@@ -3282,6 +3356,7 @@
       <c r="AG71" s="5" t="n"/>
       <c r="AH71" s="5" t="n"/>
       <c r="AI71" s="5" t="n"/>
+      <c r="AJ71" s="5" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="n"/>
@@ -3319,6 +3394,7 @@
       <c r="AG72" s="5" t="n"/>
       <c r="AH72" s="5" t="n"/>
       <c r="AI72" s="5" t="n"/>
+      <c r="AJ72" s="5" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="n"/>
@@ -3356,6 +3432,7 @@
       <c r="AG73" s="5" t="n"/>
       <c r="AH73" s="5" t="n"/>
       <c r="AI73" s="5" t="n"/>
+      <c r="AJ73" s="5" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="5" t="n"/>
@@ -3393,6 +3470,7 @@
       <c r="AG74" s="5" t="n"/>
       <c r="AH74" s="5" t="n"/>
       <c r="AI74" s="5" t="n"/>
+      <c r="AJ74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="5" t="n"/>
@@ -3430,6 +3508,7 @@
       <c r="AG75" s="5" t="n"/>
       <c r="AH75" s="5" t="n"/>
       <c r="AI75" s="5" t="n"/>
+      <c r="AJ75" s="5" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="5" t="n"/>
@@ -3467,6 +3546,7 @@
       <c r="AG76" s="5" t="n"/>
       <c r="AH76" s="5" t="n"/>
       <c r="AI76" s="5" t="n"/>
+      <c r="AJ76" s="5" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="n"/>
@@ -3504,6 +3584,7 @@
       <c r="AG77" s="5" t="n"/>
       <c r="AH77" s="5" t="n"/>
       <c r="AI77" s="5" t="n"/>
+      <c r="AJ77" s="5" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="n"/>
@@ -3541,6 +3622,7 @@
       <c r="AG78" s="5" t="n"/>
       <c r="AH78" s="5" t="n"/>
       <c r="AI78" s="5" t="n"/>
+      <c r="AJ78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="5" t="n"/>
@@ -3578,6 +3660,7 @@
       <c r="AG79" s="5" t="n"/>
       <c r="AH79" s="5" t="n"/>
       <c r="AI79" s="5" t="n"/>
+      <c r="AJ79" s="5" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="n"/>
@@ -3615,6 +3698,7 @@
       <c r="AG80" s="5" t="n"/>
       <c r="AH80" s="5" t="n"/>
       <c r="AI80" s="5" t="n"/>
+      <c r="AJ80" s="5" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="n"/>
@@ -3652,6 +3736,7 @@
       <c r="AG81" s="5" t="n"/>
       <c r="AH81" s="5" t="n"/>
       <c r="AI81" s="5" t="n"/>
+      <c r="AJ81" s="5" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="n"/>
@@ -3689,6 +3774,7 @@
       <c r="AG82" s="5" t="n"/>
       <c r="AH82" s="5" t="n"/>
       <c r="AI82" s="5" t="n"/>
+      <c r="AJ82" s="5" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="5" t="n"/>
@@ -3726,6 +3812,7 @@
       <c r="AG83" s="5" t="n"/>
       <c r="AH83" s="5" t="n"/>
       <c r="AI83" s="5" t="n"/>
+      <c r="AJ83" s="5" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="n"/>
@@ -3763,6 +3850,7 @@
       <c r="AG84" s="5" t="n"/>
       <c r="AH84" s="5" t="n"/>
       <c r="AI84" s="5" t="n"/>
+      <c r="AJ84" s="5" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="5" t="n"/>
@@ -3800,6 +3888,7 @@
       <c r="AG85" s="5" t="n"/>
       <c r="AH85" s="5" t="n"/>
       <c r="AI85" s="5" t="n"/>
+      <c r="AJ85" s="5" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="n"/>
@@ -3837,6 +3926,7 @@
       <c r="AG86" s="5" t="n"/>
       <c r="AH86" s="5" t="n"/>
       <c r="AI86" s="5" t="n"/>
+      <c r="AJ86" s="5" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="5" t="n"/>
@@ -3874,6 +3964,7 @@
       <c r="AG87" s="5" t="n"/>
       <c r="AH87" s="5" t="n"/>
       <c r="AI87" s="5" t="n"/>
+      <c r="AJ87" s="5" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="5" t="n"/>
@@ -3911,6 +4002,7 @@
       <c r="AG88" s="5" t="n"/>
       <c r="AH88" s="5" t="n"/>
       <c r="AI88" s="5" t="n"/>
+      <c r="AJ88" s="5" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="5" t="n"/>
@@ -3948,6 +4040,7 @@
       <c r="AG89" s="5" t="n"/>
       <c r="AH89" s="5" t="n"/>
       <c r="AI89" s="5" t="n"/>
+      <c r="AJ89" s="5" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="5" t="n"/>
@@ -3985,6 +4078,7 @@
       <c r="AG90" s="5" t="n"/>
       <c r="AH90" s="5" t="n"/>
       <c r="AI90" s="5" t="n"/>
+      <c r="AJ90" s="5" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="5" t="n"/>
@@ -4022,6 +4116,7 @@
       <c r="AG91" s="5" t="n"/>
       <c r="AH91" s="5" t="n"/>
       <c r="AI91" s="5" t="n"/>
+      <c r="AJ91" s="5" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="5" t="n"/>
@@ -4059,6 +4154,7 @@
       <c r="AG92" s="5" t="n"/>
       <c r="AH92" s="5" t="n"/>
       <c r="AI92" s="5" t="n"/>
+      <c r="AJ92" s="5" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="5" t="n"/>
@@ -4096,6 +4192,7 @@
       <c r="AG93" s="5" t="n"/>
       <c r="AH93" s="5" t="n"/>
       <c r="AI93" s="5" t="n"/>
+      <c r="AJ93" s="5" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="5" t="n"/>
@@ -4133,6 +4230,7 @@
       <c r="AG94" s="5" t="n"/>
       <c r="AH94" s="5" t="n"/>
       <c r="AI94" s="5" t="n"/>
+      <c r="AJ94" s="5" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="5" t="n"/>
@@ -4170,6 +4268,7 @@
       <c r="AG95" s="5" t="n"/>
       <c r="AH95" s="5" t="n"/>
       <c r="AI95" s="5" t="n"/>
+      <c r="AJ95" s="5" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="5" t="n"/>
@@ -4207,6 +4306,7 @@
       <c r="AG96" s="5" t="n"/>
       <c r="AH96" s="5" t="n"/>
       <c r="AI96" s="5" t="n"/>
+      <c r="AJ96" s="5" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="5" t="n"/>
@@ -4244,6 +4344,7 @@
       <c r="AG97" s="5" t="n"/>
       <c r="AH97" s="5" t="n"/>
       <c r="AI97" s="5" t="n"/>
+      <c r="AJ97" s="5" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="5" t="n"/>
@@ -4281,6 +4382,7 @@
       <c r="AG98" s="5" t="n"/>
       <c r="AH98" s="5" t="n"/>
       <c r="AI98" s="5" t="n"/>
+      <c r="AJ98" s="5" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="5" t="n"/>
@@ -4318,6 +4420,7 @@
       <c r="AG99" s="5" t="n"/>
       <c r="AH99" s="5" t="n"/>
       <c r="AI99" s="5" t="n"/>
+      <c r="AJ99" s="5" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="5" t="n"/>
@@ -4355,6 +4458,7 @@
       <c r="AG100" s="5" t="n"/>
       <c r="AH100" s="5" t="n"/>
       <c r="AI100" s="5" t="n"/>
+      <c r="AJ100" s="5" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="5" t="n"/>
@@ -4392,6 +4496,7 @@
       <c r="AG101" s="5" t="n"/>
       <c r="AH101" s="5" t="n"/>
       <c r="AI101" s="5" t="n"/>
+      <c r="AJ101" s="5" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="5" t="n"/>
@@ -4429,6 +4534,7 @@
       <c r="AG102" s="5" t="n"/>
       <c r="AH102" s="5" t="n"/>
       <c r="AI102" s="5" t="n"/>
+      <c r="AJ102" s="5" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="5" t="n"/>
@@ -4466,6 +4572,7 @@
       <c r="AG103" s="5" t="n"/>
       <c r="AH103" s="5" t="n"/>
       <c r="AI103" s="5" t="n"/>
+      <c r="AJ103" s="5" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="5" t="n"/>
@@ -4503,6 +4610,7 @@
       <c r="AG104" s="5" t="n"/>
       <c r="AH104" s="5" t="n"/>
       <c r="AI104" s="5" t="n"/>
+      <c r="AJ104" s="5" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="5" t="n"/>
@@ -4540,6 +4648,7 @@
       <c r="AG105" s="5" t="n"/>
       <c r="AH105" s="5" t="n"/>
       <c r="AI105" s="5" t="n"/>
+      <c r="AJ105" s="5" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="5" t="n"/>
@@ -4577,6 +4686,7 @@
       <c r="AG106" s="5" t="n"/>
       <c r="AH106" s="5" t="n"/>
       <c r="AI106" s="5" t="n"/>
+      <c r="AJ106" s="5" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="5" t="n"/>
@@ -4614,6 +4724,7 @@
       <c r="AG107" s="5" t="n"/>
       <c r="AH107" s="5" t="n"/>
       <c r="AI107" s="5" t="n"/>
+      <c r="AJ107" s="5" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="5" t="n"/>
@@ -4651,6 +4762,7 @@
       <c r="AG108" s="5" t="n"/>
       <c r="AH108" s="5" t="n"/>
       <c r="AI108" s="5" t="n"/>
+      <c r="AJ108" s="5" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="5" t="n"/>
@@ -4688,6 +4800,7 @@
       <c r="AG109" s="5" t="n"/>
       <c r="AH109" s="5" t="n"/>
       <c r="AI109" s="5" t="n"/>
+      <c r="AJ109" s="5" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="5" t="n"/>
@@ -4725,6 +4838,7 @@
       <c r="AG110" s="5" t="n"/>
       <c r="AH110" s="5" t="n"/>
       <c r="AI110" s="5" t="n"/>
+      <c r="AJ110" s="5" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="5" t="n"/>
@@ -4762,6 +4876,7 @@
       <c r="AG111" s="5" t="n"/>
       <c r="AH111" s="5" t="n"/>
       <c r="AI111" s="5" t="n"/>
+      <c r="AJ111" s="5" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="5" t="n"/>
@@ -4799,6 +4914,7 @@
       <c r="AG112" s="5" t="n"/>
       <c r="AH112" s="5" t="n"/>
       <c r="AI112" s="5" t="n"/>
+      <c r="AJ112" s="5" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="5" t="n"/>
@@ -4836,6 +4952,7 @@
       <c r="AG113" s="5" t="n"/>
       <c r="AH113" s="5" t="n"/>
       <c r="AI113" s="5" t="n"/>
+      <c r="AJ113" s="5" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="5" t="n"/>
@@ -4873,6 +4990,7 @@
       <c r="AG114" s="5" t="n"/>
       <c r="AH114" s="5" t="n"/>
       <c r="AI114" s="5" t="n"/>
+      <c r="AJ114" s="5" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="5" t="n"/>
@@ -4910,6 +5028,7 @@
       <c r="AG115" s="5" t="n"/>
       <c r="AH115" s="5" t="n"/>
       <c r="AI115" s="5" t="n"/>
+      <c r="AJ115" s="5" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="5" t="n"/>
@@ -4947,6 +5066,7 @@
       <c r="AG116" s="5" t="n"/>
       <c r="AH116" s="5" t="n"/>
       <c r="AI116" s="5" t="n"/>
+      <c r="AJ116" s="5" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="5" t="n"/>
@@ -4984,6 +5104,7 @@
       <c r="AG117" s="5" t="n"/>
       <c r="AH117" s="5" t="n"/>
       <c r="AI117" s="5" t="n"/>
+      <c r="AJ117" s="5" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="5" t="n"/>
@@ -5021,6 +5142,7 @@
       <c r="AG118" s="5" t="n"/>
       <c r="AH118" s="5" t="n"/>
       <c r="AI118" s="5" t="n"/>
+      <c r="AJ118" s="5" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="5" t="n"/>
@@ -5058,6 +5180,7 @@
       <c r="AG119" s="5" t="n"/>
       <c r="AH119" s="5" t="n"/>
       <c r="AI119" s="5" t="n"/>
+      <c r="AJ119" s="5" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="5" t="n"/>
@@ -5095,6 +5218,7 @@
       <c r="AG120" s="5" t="n"/>
       <c r="AH120" s="5" t="n"/>
       <c r="AI120" s="5" t="n"/>
+      <c r="AJ120" s="5" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="5" t="n"/>
@@ -5132,6 +5256,7 @@
       <c r="AG121" s="5" t="n"/>
       <c r="AH121" s="5" t="n"/>
       <c r="AI121" s="5" t="n"/>
+      <c r="AJ121" s="5" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="5" t="n"/>
@@ -5169,6 +5294,7 @@
       <c r="AG122" s="5" t="n"/>
       <c r="AH122" s="5" t="n"/>
       <c r="AI122" s="5" t="n"/>
+      <c r="AJ122" s="5" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="5" t="n"/>
@@ -5206,6 +5332,7 @@
       <c r="AG123" s="5" t="n"/>
       <c r="AH123" s="5" t="n"/>
       <c r="AI123" s="5" t="n"/>
+      <c r="AJ123" s="5" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="5" t="n"/>
@@ -5243,6 +5370,7 @@
       <c r="AG124" s="5" t="n"/>
       <c r="AH124" s="5" t="n"/>
       <c r="AI124" s="5" t="n"/>
+      <c r="AJ124" s="5" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="5" t="n"/>
@@ -5280,6 +5408,7 @@
       <c r="AG125" s="5" t="n"/>
       <c r="AH125" s="5" t="n"/>
       <c r="AI125" s="5" t="n"/>
+      <c r="AJ125" s="5" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="5" t="n"/>
@@ -5317,6 +5446,7 @@
       <c r="AG126" s="5" t="n"/>
       <c r="AH126" s="5" t="n"/>
       <c r="AI126" s="5" t="n"/>
+      <c r="AJ126" s="5" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="5" t="n"/>
@@ -5354,6 +5484,7 @@
       <c r="AG127" s="5" t="n"/>
       <c r="AH127" s="5" t="n"/>
       <c r="AI127" s="5" t="n"/>
+      <c r="AJ127" s="5" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="5" t="n"/>
@@ -5391,6 +5522,7 @@
       <c r="AG128" s="5" t="n"/>
       <c r="AH128" s="5" t="n"/>
       <c r="AI128" s="5" t="n"/>
+      <c r="AJ128" s="5" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="5" t="n"/>
@@ -5428,6 +5560,7 @@
       <c r="AG129" s="5" t="n"/>
       <c r="AH129" s="5" t="n"/>
       <c r="AI129" s="5" t="n"/>
+      <c r="AJ129" s="5" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="5" t="n"/>
@@ -5465,6 +5598,7 @@
       <c r="AG130" s="5" t="n"/>
       <c r="AH130" s="5" t="n"/>
       <c r="AI130" s="5" t="n"/>
+      <c r="AJ130" s="5" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="5" t="n"/>
@@ -5502,6 +5636,7 @@
       <c r="AG131" s="5" t="n"/>
       <c r="AH131" s="5" t="n"/>
       <c r="AI131" s="5" t="n"/>
+      <c r="AJ131" s="5" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="5" t="n"/>
@@ -5539,6 +5674,7 @@
       <c r="AG132" s="5" t="n"/>
       <c r="AH132" s="5" t="n"/>
       <c r="AI132" s="5" t="n"/>
+      <c r="AJ132" s="5" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="5" t="n"/>
@@ -5576,6 +5712,7 @@
       <c r="AG133" s="5" t="n"/>
       <c r="AH133" s="5" t="n"/>
       <c r="AI133" s="5" t="n"/>
+      <c r="AJ133" s="5" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="5" t="n"/>
@@ -5613,6 +5750,7 @@
       <c r="AG134" s="5" t="n"/>
       <c r="AH134" s="5" t="n"/>
       <c r="AI134" s="5" t="n"/>
+      <c r="AJ134" s="5" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="5" t="n"/>
@@ -5650,6 +5788,7 @@
       <c r="AG135" s="5" t="n"/>
       <c r="AH135" s="5" t="n"/>
       <c r="AI135" s="5" t="n"/>
+      <c r="AJ135" s="5" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="5" t="n"/>
@@ -5687,6 +5826,7 @@
       <c r="AG136" s="5" t="n"/>
       <c r="AH136" s="5" t="n"/>
       <c r="AI136" s="5" t="n"/>
+      <c r="AJ136" s="5" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="5" t="n"/>
@@ -5724,6 +5864,7 @@
       <c r="AG137" s="5" t="n"/>
       <c r="AH137" s="5" t="n"/>
       <c r="AI137" s="5" t="n"/>
+      <c r="AJ137" s="5" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="5" t="n"/>
@@ -5761,6 +5902,7 @@
       <c r="AG138" s="5" t="n"/>
       <c r="AH138" s="5" t="n"/>
       <c r="AI138" s="5" t="n"/>
+      <c r="AJ138" s="5" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="5" t="n"/>
@@ -5798,6 +5940,7 @@
       <c r="AG139" s="5" t="n"/>
       <c r="AH139" s="5" t="n"/>
       <c r="AI139" s="5" t="n"/>
+      <c r="AJ139" s="5" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="5" t="n"/>
@@ -5835,6 +5978,7 @@
       <c r="AG140" s="5" t="n"/>
       <c r="AH140" s="5" t="n"/>
       <c r="AI140" s="5" t="n"/>
+      <c r="AJ140" s="5" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="5" t="n"/>
@@ -5872,6 +6016,7 @@
       <c r="AG141" s="5" t="n"/>
       <c r="AH141" s="5" t="n"/>
       <c r="AI141" s="5" t="n"/>
+      <c r="AJ141" s="5" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="5" t="n"/>
@@ -5909,6 +6054,7 @@
       <c r="AG142" s="5" t="n"/>
       <c r="AH142" s="5" t="n"/>
       <c r="AI142" s="5" t="n"/>
+      <c r="AJ142" s="5" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="5" t="n"/>
@@ -5946,6 +6092,7 @@
       <c r="AG143" s="5" t="n"/>
       <c r="AH143" s="5" t="n"/>
       <c r="AI143" s="5" t="n"/>
+      <c r="AJ143" s="5" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="5" t="n"/>
@@ -5983,6 +6130,7 @@
       <c r="AG144" s="5" t="n"/>
       <c r="AH144" s="5" t="n"/>
       <c r="AI144" s="5" t="n"/>
+      <c r="AJ144" s="5" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="5" t="n"/>
@@ -6020,6 +6168,7 @@
       <c r="AG145" s="5" t="n"/>
       <c r="AH145" s="5" t="n"/>
       <c r="AI145" s="5" t="n"/>
+      <c r="AJ145" s="5" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="5" t="n"/>
@@ -6057,6 +6206,7 @@
       <c r="AG146" s="5" t="n"/>
       <c r="AH146" s="5" t="n"/>
       <c r="AI146" s="5" t="n"/>
+      <c r="AJ146" s="5" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="5" t="n"/>
@@ -6094,6 +6244,7 @@
       <c r="AG147" s="5" t="n"/>
       <c r="AH147" s="5" t="n"/>
       <c r="AI147" s="5" t="n"/>
+      <c r="AJ147" s="5" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="5" t="n"/>
@@ -6131,6 +6282,7 @@
       <c r="AG148" s="5" t="n"/>
       <c r="AH148" s="5" t="n"/>
       <c r="AI148" s="5" t="n"/>
+      <c r="AJ148" s="5" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="5" t="n"/>
@@ -6168,6 +6320,7 @@
       <c r="AG149" s="5" t="n"/>
       <c r="AH149" s="5" t="n"/>
       <c r="AI149" s="5" t="n"/>
+      <c r="AJ149" s="5" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="5" t="n"/>
@@ -6205,6 +6358,7 @@
       <c r="AG150" s="5" t="n"/>
       <c r="AH150" s="5" t="n"/>
       <c r="AI150" s="5" t="n"/>
+      <c r="AJ150" s="5" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="5" t="n"/>
@@ -6242,6 +6396,7 @@
       <c r="AG151" s="5" t="n"/>
       <c r="AH151" s="5" t="n"/>
       <c r="AI151" s="5" t="n"/>
+      <c r="AJ151" s="5" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="5" t="n"/>
@@ -6279,6 +6434,7 @@
       <c r="AG152" s="5" t="n"/>
       <c r="AH152" s="5" t="n"/>
       <c r="AI152" s="5" t="n"/>
+      <c r="AJ152" s="5" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="5" t="n"/>
@@ -6316,6 +6472,7 @@
       <c r="AG153" s="5" t="n"/>
       <c r="AH153" s="5" t="n"/>
       <c r="AI153" s="5" t="n"/>
+      <c r="AJ153" s="5" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="5" t="n"/>
@@ -6353,6 +6510,7 @@
       <c r="AG154" s="5" t="n"/>
       <c r="AH154" s="5" t="n"/>
       <c r="AI154" s="5" t="n"/>
+      <c r="AJ154" s="5" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="5" t="n"/>
@@ -6390,6 +6548,7 @@
       <c r="AG155" s="5" t="n"/>
       <c r="AH155" s="5" t="n"/>
       <c r="AI155" s="5" t="n"/>
+      <c r="AJ155" s="5" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="5" t="n"/>
@@ -6427,6 +6586,7 @@
       <c r="AG156" s="5" t="n"/>
       <c r="AH156" s="5" t="n"/>
       <c r="AI156" s="5" t="n"/>
+      <c r="AJ156" s="5" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="5" t="n"/>
@@ -6464,6 +6624,7 @@
       <c r="AG157" s="5" t="n"/>
       <c r="AH157" s="5" t="n"/>
       <c r="AI157" s="5" t="n"/>
+      <c r="AJ157" s="5" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="5" t="n"/>
@@ -6501,6 +6662,7 @@
       <c r="AG158" s="5" t="n"/>
       <c r="AH158" s="5" t="n"/>
       <c r="AI158" s="5" t="n"/>
+      <c r="AJ158" s="5" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="5" t="n"/>
@@ -6538,6 +6700,7 @@
       <c r="AG159" s="5" t="n"/>
       <c r="AH159" s="5" t="n"/>
       <c r="AI159" s="5" t="n"/>
+      <c r="AJ159" s="5" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="5" t="n"/>
@@ -6575,6 +6738,7 @@
       <c r="AG160" s="5" t="n"/>
       <c r="AH160" s="5" t="n"/>
       <c r="AI160" s="5" t="n"/>
+      <c r="AJ160" s="5" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="5" t="n"/>
@@ -6612,6 +6776,7 @@
       <c r="AG161" s="5" t="n"/>
       <c r="AH161" s="5" t="n"/>
       <c r="AI161" s="5" t="n"/>
+      <c r="AJ161" s="5" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="5" t="n"/>
@@ -6649,6 +6814,7 @@
       <c r="AG162" s="5" t="n"/>
       <c r="AH162" s="5" t="n"/>
       <c r="AI162" s="5" t="n"/>
+      <c r="AJ162" s="5" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="5" t="n"/>
@@ -6686,6 +6852,7 @@
       <c r="AG163" s="5" t="n"/>
       <c r="AH163" s="5" t="n"/>
       <c r="AI163" s="5" t="n"/>
+      <c r="AJ163" s="5" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="5" t="n"/>
@@ -6723,6 +6890,7 @@
       <c r="AG164" s="5" t="n"/>
       <c r="AH164" s="5" t="n"/>
       <c r="AI164" s="5" t="n"/>
+      <c r="AJ164" s="5" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="5" t="n"/>
@@ -6760,6 +6928,7 @@
       <c r="AG165" s="5" t="n"/>
       <c r="AH165" s="5" t="n"/>
       <c r="AI165" s="5" t="n"/>
+      <c r="AJ165" s="5" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="5" t="n"/>
@@ -6797,6 +6966,7 @@
       <c r="AG166" s="5" t="n"/>
       <c r="AH166" s="5" t="n"/>
       <c r="AI166" s="5" t="n"/>
+      <c r="AJ166" s="5" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="5" t="n"/>
@@ -6834,6 +7004,7 @@
       <c r="AG167" s="5" t="n"/>
       <c r="AH167" s="5" t="n"/>
       <c r="AI167" s="5" t="n"/>
+      <c r="AJ167" s="5" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="5" t="n"/>
@@ -6871,6 +7042,7 @@
       <c r="AG168" s="5" t="n"/>
       <c r="AH168" s="5" t="n"/>
       <c r="AI168" s="5" t="n"/>
+      <c r="AJ168" s="5" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="5" t="n"/>
@@ -6908,6 +7080,7 @@
       <c r="AG169" s="5" t="n"/>
       <c r="AH169" s="5" t="n"/>
       <c r="AI169" s="5" t="n"/>
+      <c r="AJ169" s="5" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="5" t="n"/>
@@ -6945,6 +7118,7 @@
       <c r="AG170" s="5" t="n"/>
       <c r="AH170" s="5" t="n"/>
       <c r="AI170" s="5" t="n"/>
+      <c r="AJ170" s="5" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="5" t="n"/>
@@ -6982,6 +7156,7 @@
       <c r="AG171" s="5" t="n"/>
       <c r="AH171" s="5" t="n"/>
       <c r="AI171" s="5" t="n"/>
+      <c r="AJ171" s="5" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="5" t="n"/>
@@ -7019,6 +7194,7 @@
       <c r="AG172" s="5" t="n"/>
       <c r="AH172" s="5" t="n"/>
       <c r="AI172" s="5" t="n"/>
+      <c r="AJ172" s="5" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="5" t="n"/>
@@ -7056,6 +7232,7 @@
       <c r="AG173" s="5" t="n"/>
       <c r="AH173" s="5" t="n"/>
       <c r="AI173" s="5" t="n"/>
+      <c r="AJ173" s="5" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="5" t="n"/>
@@ -7093,6 +7270,7 @@
       <c r="AG174" s="5" t="n"/>
       <c r="AH174" s="5" t="n"/>
       <c r="AI174" s="5" t="n"/>
+      <c r="AJ174" s="5" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="5" t="n"/>
@@ -7130,6 +7308,7 @@
       <c r="AG175" s="5" t="n"/>
       <c r="AH175" s="5" t="n"/>
       <c r="AI175" s="5" t="n"/>
+      <c r="AJ175" s="5" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="5" t="n"/>
@@ -7167,6 +7346,7 @@
       <c r="AG176" s="5" t="n"/>
       <c r="AH176" s="5" t="n"/>
       <c r="AI176" s="5" t="n"/>
+      <c r="AJ176" s="5" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="5" t="n"/>
@@ -7204,6 +7384,7 @@
       <c r="AG177" s="5" t="n"/>
       <c r="AH177" s="5" t="n"/>
       <c r="AI177" s="5" t="n"/>
+      <c r="AJ177" s="5" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="5" t="n"/>
@@ -7241,6 +7422,7 @@
       <c r="AG178" s="5" t="n"/>
       <c r="AH178" s="5" t="n"/>
       <c r="AI178" s="5" t="n"/>
+      <c r="AJ178" s="5" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="5" t="n"/>
@@ -7278,6 +7460,7 @@
       <c r="AG179" s="5" t="n"/>
       <c r="AH179" s="5" t="n"/>
       <c r="AI179" s="5" t="n"/>
+      <c r="AJ179" s="5" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="5" t="n"/>
@@ -7315,6 +7498,7 @@
       <c r="AG180" s="5" t="n"/>
       <c r="AH180" s="5" t="n"/>
       <c r="AI180" s="5" t="n"/>
+      <c r="AJ180" s="5" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="5" t="n"/>
@@ -7352,6 +7536,7 @@
       <c r="AG181" s="5" t="n"/>
       <c r="AH181" s="5" t="n"/>
       <c r="AI181" s="5" t="n"/>
+      <c r="AJ181" s="5" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="5" t="n"/>
@@ -7389,6 +7574,7 @@
       <c r="AG182" s="5" t="n"/>
       <c r="AH182" s="5" t="n"/>
       <c r="AI182" s="5" t="n"/>
+      <c r="AJ182" s="5" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="5" t="n"/>
@@ -7426,6 +7612,7 @@
       <c r="AG183" s="5" t="n"/>
       <c r="AH183" s="5" t="n"/>
       <c r="AI183" s="5" t="n"/>
+      <c r="AJ183" s="5" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="5" t="n"/>
@@ -7463,6 +7650,7 @@
       <c r="AG184" s="5" t="n"/>
       <c r="AH184" s="5" t="n"/>
       <c r="AI184" s="5" t="n"/>
+      <c r="AJ184" s="5" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="5" t="n"/>
@@ -7500,6 +7688,7 @@
       <c r="AG185" s="5" t="n"/>
       <c r="AH185" s="5" t="n"/>
       <c r="AI185" s="5" t="n"/>
+      <c r="AJ185" s="5" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="5" t="n"/>
@@ -7537,6 +7726,7 @@
       <c r="AG186" s="5" t="n"/>
       <c r="AH186" s="5" t="n"/>
       <c r="AI186" s="5" t="n"/>
+      <c r="AJ186" s="5" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="5" t="n"/>
@@ -7574,6 +7764,7 @@
       <c r="AG187" s="5" t="n"/>
       <c r="AH187" s="5" t="n"/>
       <c r="AI187" s="5" t="n"/>
+      <c r="AJ187" s="5" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="5" t="n"/>
@@ -7611,6 +7802,7 @@
       <c r="AG188" s="5" t="n"/>
       <c r="AH188" s="5" t="n"/>
       <c r="AI188" s="5" t="n"/>
+      <c r="AJ188" s="5" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="5" t="n"/>
@@ -7648,6 +7840,7 @@
       <c r="AG189" s="5" t="n"/>
       <c r="AH189" s="5" t="n"/>
       <c r="AI189" s="5" t="n"/>
+      <c r="AJ189" s="5" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="5" t="n"/>
@@ -7685,6 +7878,7 @@
       <c r="AG190" s="5" t="n"/>
       <c r="AH190" s="5" t="n"/>
       <c r="AI190" s="5" t="n"/>
+      <c r="AJ190" s="5" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="5" t="n"/>
@@ -7722,6 +7916,7 @@
       <c r="AG191" s="5" t="n"/>
       <c r="AH191" s="5" t="n"/>
       <c r="AI191" s="5" t="n"/>
+      <c r="AJ191" s="5" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="5" t="n"/>
@@ -7759,6 +7954,7 @@
       <c r="AG192" s="5" t="n"/>
       <c r="AH192" s="5" t="n"/>
       <c r="AI192" s="5" t="n"/>
+      <c r="AJ192" s="5" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="5" t="n"/>
@@ -7796,6 +7992,7 @@
       <c r="AG193" s="5" t="n"/>
       <c r="AH193" s="5" t="n"/>
       <c r="AI193" s="5" t="n"/>
+      <c r="AJ193" s="5" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="5" t="n"/>
@@ -7833,6 +8030,7 @@
       <c r="AG194" s="5" t="n"/>
       <c r="AH194" s="5" t="n"/>
       <c r="AI194" s="5" t="n"/>
+      <c r="AJ194" s="5" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="5" t="n"/>
@@ -7870,6 +8068,7 @@
       <c r="AG195" s="5" t="n"/>
       <c r="AH195" s="5" t="n"/>
       <c r="AI195" s="5" t="n"/>
+      <c r="AJ195" s="5" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="5" t="n"/>
@@ -7907,6 +8106,7 @@
       <c r="AG196" s="5" t="n"/>
       <c r="AH196" s="5" t="n"/>
       <c r="AI196" s="5" t="n"/>
+      <c r="AJ196" s="5" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="5" t="n"/>
@@ -7944,6 +8144,7 @@
       <c r="AG197" s="5" t="n"/>
       <c r="AH197" s="5" t="n"/>
       <c r="AI197" s="5" t="n"/>
+      <c r="AJ197" s="5" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="5" t="n"/>
@@ -7981,6 +8182,7 @@
       <c r="AG198" s="5" t="n"/>
       <c r="AH198" s="5" t="n"/>
       <c r="AI198" s="5" t="n"/>
+      <c r="AJ198" s="5" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="5" t="n"/>
@@ -8018,6 +8220,7 @@
       <c r="AG199" s="5" t="n"/>
       <c r="AH199" s="5" t="n"/>
       <c r="AI199" s="5" t="n"/>
+      <c r="AJ199" s="5" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="5" t="n"/>
@@ -8055,12 +8258,13 @@
       <c r="AG200" s="5" t="n"/>
       <c r="AH200" s="5" t="n"/>
       <c r="AI200" s="5" t="n"/>
+      <c r="AJ200" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="T1:AI1"/>
     <mergeCell ref="A1:O1"/>
-    <mergeCell ref="P1:S1"/>
+    <mergeCell ref="U1:AJ1"/>
+    <mergeCell ref="P1:T1"/>
   </mergeCells>
   <dataValidations count="11">
     <dataValidation sqref="C3:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -8075,25 +8279,25 @@
     <dataValidation sqref="P3:P200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lists!$D$2:$D$4</formula1>
     </dataValidation>
-    <dataValidation sqref="V3:V200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="W3:W200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lists!$E$2:$E$3</formula1>
     </dataValidation>
-    <dataValidation sqref="X3:X200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Y3:Y200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lists!$F$2:$F$3</formula1>
     </dataValidation>
-    <dataValidation sqref="Y3:Y200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Z3:Z200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lists!$G$2:$G$3</formula1>
     </dataValidation>
-    <dataValidation sqref="AC3:AC200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AD3:AD200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lists!$H$2:$H$3</formula1>
     </dataValidation>
-    <dataValidation sqref="AF3:AF200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AG3:AG200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lists!$I$2:$I$3</formula1>
     </dataValidation>
-    <dataValidation sqref="AG3:AG200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AH3:AH200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lists!$J$2:$J$3</formula1>
     </dataValidation>
-    <dataValidation sqref="AI3:AI200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AJ3:AJ200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_lists!$K$2:$K$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>